<commit_message>
Rebuild candidate-visible task contract
</commit_message>
<xml_diff>
--- a/artifacts/任务规格转化.xlsx
+++ b/artifacts/任务规格转化.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="任务规格转化" sheetId="1" r:id="R749cffc6ee494432"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="任务规格转化" sheetId="1" r:id="Ree45017c89ce4ed4"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -371,7 +371,7 @@
         <x:v>核心操作链</x:v>
       </x:c>
       <x:c r="B9" s="7" t="str">
-        <x:v>排序申请；规范化URL；重建UTM；识别现网占用；处置短码；生成映射；汇总迁移</x:v>
+        <x:v>排序申请；规整URL；重建UTM；识别现网占用；处置短码；生成映射；汇总迁移</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="32" customHeight="1">
@@ -384,10 +384,10 @@
     </x:row>
     <x:row r="11" ht="32" customHeight="1">
       <x:c r="A11" s="7" t="str">
-        <x:v>短码裁决</x:v>
+        <x:v>短码处置</x:v>
       </x:c>
       <x:c r="B11" s="7" t="str">
-        <x:v>按run_at_utc区分占用和回收，复用需要团队与规范化目标同时一致，冲突使用最小可用后缀</x:v>
+        <x:v>按run_at_utc区分占用和收回，沿用需要团队与规整后目标同时一致，冲突使用最小可用后缀</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="46" customHeight="1">
@@ -408,10 +408,10 @@
     </x:row>
     <x:row r="14" ht="32" customHeight="1">
       <x:c r="A14" s="7" t="str">
-        <x:v>汇总合同</x:v>
+        <x:v>迁移汇总</x:v>
       </x:c>
       <x:c r="B14" s="7" t="str">
-        <x:v>migration_summary.json从处置记录和路由映射复算主要迁移分支</x:v>
+        <x:v>migration_summary.json从处置记录和路由映射汇总主要处置分支</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="32" customHeight="1">
@@ -419,7 +419,7 @@
         <x:v>完成条件</x:v>
       </x:c>
       <x:c r="B15" s="7" t="str">
-        <x:v>Node.js入口正常结束，四份交付可读，request_id与slug能够跨文件追溯，汇总数量闭合</x:v>
+        <x:v>Node.js入口正常结束，四份交付可读，request_id与slug能够跨文件对应，汇总数量相互一致</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="32" customHeight="1">
@@ -427,7 +427,7 @@
         <x:v>可验证点</x:v>
       </x:c>
       <x:c r="B16" s="7" t="str">
-        <x:v>协议、域名、query键、UTM、短码状态、处置身份和汇总均能从输入复算</x:v>
+        <x:v>协议、域名、query字段、UTM、短码状态、处置结论和汇总均能从输入对应</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="32" customHeight="1">

</xml_diff>